<commit_message>
Publish Racice_2022_WC, Montemor_2025_JWCH, Auronzo_2023_JWCH
</commit_message>
<xml_diff>
--- a/events/Racice_2022_WC/Racice_2022_WC_Results.xlsx
+++ b/events/Racice_2022_WC/Racice_2022_WC_Results.xlsx
@@ -2627,6 +2627,11 @@
           <t>42426</t>
         </is>
       </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>42425</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2877,6 +2882,11 @@
           <t>65694</t>
         </is>
       </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>97652</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3362,6 +3372,11 @@
           <t>97611</t>
         </is>
       </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>97631</t>
+        </is>
+      </c>
       <c r="T37" t="inlineStr">
         <is>
           <t>88695</t>
@@ -4197,6 +4212,11 @@
           <t>118805</t>
         </is>
       </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>97726</t>
+        </is>
+      </c>
       <c r="U47" t="inlineStr">
         <is>
           <t>118804</t>
@@ -5537,6 +5557,11 @@
           <t>111737</t>
         </is>
       </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>97656</t>
+        </is>
+      </c>
       <c r="U63" t="inlineStr">
         <is>
           <t>111736</t>
@@ -8422,6 +8447,11 @@
           <t>+3.556</t>
         </is>
       </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>97902</t>
+        </is>
+      </c>
       <c r="S102" t="inlineStr">
         <is>
           <t>50167</t>
@@ -8797,6 +8827,11 @@
           <t>105031</t>
         </is>
       </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>97732</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -9692,6 +9727,11 @@
           <t>+5.453</t>
         </is>
       </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>97723</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -11752,6 +11792,11 @@
           <t>+4.074</t>
         </is>
       </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>42517</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -18100,6 +18145,11 @@
           <t>+11.678</t>
         </is>
       </c>
+      <c r="R242" t="inlineStr">
+        <is>
+          <t>97723</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -19310,6 +19360,11 @@
           <t>42426</t>
         </is>
       </c>
+      <c r="U259" t="inlineStr">
+        <is>
+          <t>42425</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -20395,6 +20450,11 @@
           <t>65694</t>
         </is>
       </c>
+      <c r="U272" t="inlineStr">
+        <is>
+          <t>97652</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -21730,6 +21790,11 @@
           <t>118805</t>
         </is>
       </c>
+      <c r="T289" t="inlineStr">
+        <is>
+          <t>97726</t>
+        </is>
+      </c>
       <c r="U289" t="inlineStr">
         <is>
           <t>118804</t>
@@ -23230,6 +23295,11 @@
           <t>97611</t>
         </is>
       </c>
+      <c r="S307" t="inlineStr">
+        <is>
+          <t>97631</t>
+        </is>
+      </c>
       <c r="T307" t="inlineStr">
         <is>
           <t>88695</t>
@@ -23400,6 +23470,11 @@
           <t>111737</t>
         </is>
       </c>
+      <c r="T309" t="inlineStr">
+        <is>
+          <t>97656</t>
+        </is>
+      </c>
       <c r="U309" t="inlineStr">
         <is>
           <t>111736</t>
@@ -23625,6 +23700,11 @@
           <t>+0.870</t>
         </is>
       </c>
+      <c r="R312" t="inlineStr">
+        <is>
+          <t>97902</t>
+        </is>
+      </c>
       <c r="S312" t="inlineStr">
         <is>
           <t>50167</t>
@@ -26540,6 +26620,11 @@
           <t>+6.860</t>
         </is>
       </c>
+      <c r="R353" t="inlineStr">
+        <is>
+          <t>97723</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -28405,6 +28490,11 @@
           <t>+4.707</t>
         </is>
       </c>
+      <c r="R380" t="inlineStr">
+        <is>
+          <t>42517</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -35783,6 +35873,11 @@
       <c r="L487" t="n">
         <v>2</v>
       </c>
+      <c r="R487" t="inlineStr">
+        <is>
+          <t>97732</t>
+        </is>
+      </c>
       <c r="X487" t="inlineStr">
         <is>
           <t>DSQ</t>
@@ -36468,6 +36563,11 @@
           <t>+3.310</t>
         </is>
       </c>
+      <c r="R497" t="inlineStr">
+        <is>
+          <t>97902</t>
+        </is>
+      </c>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
@@ -38168,6 +38268,11 @@
           <t>+0.413</t>
         </is>
       </c>
+      <c r="R521" t="inlineStr">
+        <is>
+          <t>97656</t>
+        </is>
+      </c>
       <c r="S521" t="inlineStr">
         <is>
           <t>77253</t>
@@ -39503,6 +39608,11 @@
           <t>+8.804</t>
         </is>
       </c>
+      <c r="R540" t="inlineStr">
+        <is>
+          <t>97652</t>
+        </is>
+      </c>
     </row>
     <row r="541">
       <c r="A541" t="inlineStr">
@@ -39983,6 +40093,11 @@
           <t>+5.217</t>
         </is>
       </c>
+      <c r="R547" t="inlineStr">
+        <is>
+          <t>42517</t>
+        </is>
+      </c>
     </row>
     <row r="548">
       <c r="A548" t="inlineStr">
@@ -40809,6 +40924,11 @@
           <t>65694</t>
         </is>
       </c>
+      <c r="U557" t="inlineStr">
+        <is>
+          <t>97652</t>
+        </is>
+      </c>
     </row>
     <row r="558">
       <c r="A558" t="inlineStr">
@@ -41567,6 +41687,11 @@
           <t>118805</t>
         </is>
       </c>
+      <c r="T566" t="inlineStr">
+        <is>
+          <t>97726</t>
+        </is>
+      </c>
       <c r="U566" t="inlineStr">
         <is>
           <t>118804</t>
@@ -41644,6 +41769,11 @@
           <t>97611</t>
         </is>
       </c>
+      <c r="S567" t="inlineStr">
+        <is>
+          <t>97631</t>
+        </is>
+      </c>
       <c r="T567" t="inlineStr">
         <is>
           <t>88695</t>
@@ -43176,6 +43306,11 @@
           <t>+1.064</t>
         </is>
       </c>
+      <c r="R588" t="inlineStr">
+        <is>
+          <t>42517</t>
+        </is>
+      </c>
     </row>
     <row r="589">
       <c r="A589" t="inlineStr">
@@ -47263,6 +47398,11 @@
           <t>42426</t>
         </is>
       </c>
+      <c r="U644" t="inlineStr">
+        <is>
+          <t>42425</t>
+        </is>
+      </c>
     </row>
     <row r="645">
       <c r="A645" t="inlineStr">
@@ -49561,6 +49701,11 @@
           <t>+2.683</t>
         </is>
       </c>
+      <c r="R673" t="inlineStr">
+        <is>
+          <t>97902</t>
+        </is>
+      </c>
       <c r="S673" t="inlineStr">
         <is>
           <t>50167</t>
@@ -56869,6 +57014,11 @@
           <t>+1.733</t>
         </is>
       </c>
+      <c r="R775" t="inlineStr">
+        <is>
+          <t>42425</t>
+        </is>
+      </c>
       <c r="S775" t="inlineStr">
         <is>
           <t>39777</t>
@@ -58864,6 +59014,11 @@
           <t>+1.883</t>
         </is>
       </c>
+      <c r="R802" t="inlineStr">
+        <is>
+          <t>42724</t>
+        </is>
+      </c>
       <c r="S802" t="inlineStr">
         <is>
           <t>42728</t>
@@ -60344,6 +60499,11 @@
           <t>118805</t>
         </is>
       </c>
+      <c r="S822" t="inlineStr">
+        <is>
+          <t>97726</t>
+        </is>
+      </c>
     </row>
     <row r="823">
       <c r="A823" t="inlineStr">
@@ -64439,6 +64599,11 @@
           <t>+2.747</t>
         </is>
       </c>
+      <c r="R880" t="inlineStr">
+        <is>
+          <t>97902</t>
+        </is>
+      </c>
     </row>
     <row r="881">
       <c r="A881" t="inlineStr">
@@ -67099,6 +67264,11 @@
           <t>+9.324</t>
         </is>
       </c>
+      <c r="R918" t="inlineStr">
+        <is>
+          <t>42517</t>
+        </is>
+      </c>
     </row>
     <row r="919">
       <c r="A919" t="inlineStr">
@@ -67164,6 +67334,11 @@
           <t>+9.807</t>
         </is>
       </c>
+      <c r="R919" t="inlineStr">
+        <is>
+          <t>97652</t>
+        </is>
+      </c>
     </row>
     <row r="920">
       <c r="A920" t="inlineStr">
@@ -70224,6 +70399,11 @@
           <t>+3.507</t>
         </is>
       </c>
+      <c r="R962" t="inlineStr">
+        <is>
+          <t>42425</t>
+        </is>
+      </c>
       <c r="S962" t="inlineStr">
         <is>
           <t>39777</t>
@@ -73559,6 +73739,11 @@
           <t>+3.430</t>
         </is>
       </c>
+      <c r="R1007" t="inlineStr">
+        <is>
+          <t>97732</t>
+        </is>
+      </c>
       <c r="S1007" t="inlineStr">
         <is>
           <t>75588</t>
@@ -75404,6 +75589,11 @@
           <t>1:48.283</t>
         </is>
       </c>
+      <c r="R1032" t="inlineStr">
+        <is>
+          <t>97732</t>
+        </is>
+      </c>
       <c r="S1032" t="inlineStr">
         <is>
           <t>75588</t>
@@ -77797,6 +77987,11 @@
           <t>3:57.458</t>
         </is>
       </c>
+      <c r="R1065" t="inlineStr">
+        <is>
+          <t>97902</t>
+        </is>
+      </c>
     </row>
     <row r="1066">
       <c r="A1066" t="inlineStr">
@@ -79633,6 +79828,11 @@
           <t>1:44.486</t>
         </is>
       </c>
+      <c r="R1091" t="inlineStr">
+        <is>
+          <t>42425</t>
+        </is>
+      </c>
       <c r="S1091" t="inlineStr">
         <is>
           <t>39777</t>
@@ -83909,6 +84109,11 @@
           <t>+3.104</t>
         </is>
       </c>
+      <c r="R1149" t="inlineStr">
+        <is>
+          <t>97656</t>
+        </is>
+      </c>
       <c r="S1149" t="inlineStr">
         <is>
           <t>77253</t>
@@ -88075,6 +88280,11 @@
           <t>+5.833</t>
         </is>
       </c>
+      <c r="R1205" t="inlineStr">
+        <is>
+          <t>97732</t>
+        </is>
+      </c>
       <c r="S1205" t="inlineStr">
         <is>
           <t>75588</t>
@@ -90310,6 +90520,11 @@
           <t>+1:46.645</t>
         </is>
       </c>
+      <c r="R1236" t="inlineStr">
+        <is>
+          <t>97902</t>
+        </is>
+      </c>
     </row>
     <row r="1237">
       <c r="A1237" t="inlineStr">
@@ -93570,6 +93785,11 @@
           <t>+1:15.026</t>
         </is>
       </c>
+      <c r="R1284" t="inlineStr">
+        <is>
+          <t>42724</t>
+        </is>
+      </c>
     </row>
     <row r="1285">
       <c r="A1285" t="inlineStr">
@@ -94470,6 +94690,11 @@
       </c>
       <c r="N1297" t="n">
         <v>27</v>
+      </c>
+      <c r="R1297" t="inlineStr">
+        <is>
+          <t>97723</t>
+        </is>
       </c>
     </row>
     <row r="1298">
@@ -94912,7 +95137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D490"/>
+  <dimension ref="A1:D500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -105695,6 +105920,226 @@
         </is>
       </c>
     </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>42425</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Agata</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>FANTINI</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>97652</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Anna</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>HANSEN</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>97631</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Mark</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>SZENDY</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>97726</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Taehyeon</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>KIM</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>97656</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Philip</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>BRYDE</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>97902</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Gabriele</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>CASADEI</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>97732</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Mihai</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>CHIHAIA</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>97723</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Gihong</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>GWON</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>42517</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Esti</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>OLIVIER</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>42724</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>DAL BO</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>